<commit_message>
feat(catalog): auto preliminary review for ZY gallery cards
Strict auto-approve existing/new candidates, mark needs_review/rejected,
update decisions JSON/Excel and gallery filters. No production changes.

Co-authored-by: sharipdaitmirzaev-hue <sharipdaitmirzaev-hue@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/imports/zelenoe-yabloko-images/review-decisions.xlsx
+++ b/data/imports/zelenoe-yabloko-images/review-decisions.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P49"/>
+  <dimension ref="A1:U49"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -449,6 +449,21 @@
       <c r="P1" t="str">
         <v>sha256</v>
       </c>
+      <c r="Q1" t="str">
+        <v>auto_reviewed</v>
+      </c>
+      <c r="R1" t="str">
+        <v>auto_review_confidence</v>
+      </c>
+      <c r="S1" t="str">
+        <v>matched_features</v>
+      </c>
+      <c r="T1" t="str">
+        <v>mismatches</v>
+      </c>
+      <c r="U1" t="str">
+        <v>decision_reason</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2">
@@ -472,9 +487,6 @@
       <c r="G2" t="str">
         <v>unknown</v>
       </c>
-      <c r="H2" t="str">
-        <v/>
-      </c>
       <c r="I2" t="str">
         <v/>
       </c>
@@ -485,10 +497,10 @@
         <v/>
       </c>
       <c r="L2" t="str">
-        <v>pending</v>
+        <v>needs_review</v>
       </c>
       <c r="M2" t="str">
-        <v/>
+        <v>Авто: статус unknown требует ручной проверки</v>
       </c>
       <c r="N2">
         <v>1254</v>
@@ -498,6 +510,21 @@
       </c>
       <c r="P2" t="str">
         <v>638c282f5311bdf8ff5043911f7c57b1289a684bd97bbfb730d2e545492fded8</v>
+      </c>
+      <c r="Q2" t="b">
+        <v>1</v>
+      </c>
+      <c r="R2">
+        <v>0.55</v>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v>status_unknown</v>
+      </c>
+      <c r="U2" t="str">
+        <v>needs_review_unknown</v>
       </c>
     </row>
     <row r="3">
@@ -522,9 +549,6 @@
       <c r="G3" t="str">
         <v>new_product</v>
       </c>
-      <c r="H3" t="str">
-        <v/>
-      </c>
       <c r="I3" t="str">
         <v/>
       </c>
@@ -535,10 +559,10 @@
         <v/>
       </c>
       <c r="L3" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M3" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KAZBEGI-2000-PET-001. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N3">
         <v>800</v>
@@ -548,6 +572,21 @@
       </c>
       <c r="P3" t="str">
         <v>6b5a6a16a6ce1ad35953d32152ca22964c8a18ce3751bc11c6edec8f8ebe0a9e</v>
+      </c>
+      <c r="Q3" t="b">
+        <v>1</v>
+      </c>
+      <c r="R3">
+        <v>0.78</v>
+      </c>
+      <c r="S3" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="4">
@@ -572,9 +611,6 @@
       <c r="G4" t="str">
         <v>new_product</v>
       </c>
-      <c r="H4" t="str">
-        <v/>
-      </c>
       <c r="I4" t="str">
         <v/>
       </c>
@@ -585,10 +621,10 @@
         <v/>
       </c>
       <c r="L4" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M4" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KAZBEGI-2000-PET-002. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N4">
         <v>600</v>
@@ -598,6 +634,21 @@
       </c>
       <c r="P4" t="str">
         <v>8590762f8239cd42913720ed9ca6f387de1c44738e3876dda7d5e14d9b5a51d2</v>
+      </c>
+      <c r="Q4" t="b">
+        <v>1</v>
+      </c>
+      <c r="R4">
+        <v>0.78</v>
+      </c>
+      <c r="S4" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="5">
@@ -622,9 +673,6 @@
       <c r="G5" t="str">
         <v>new_product</v>
       </c>
-      <c r="H5" t="str">
-        <v/>
-      </c>
       <c r="I5" t="str">
         <v/>
       </c>
@@ -635,10 +683,10 @@
         <v/>
       </c>
       <c r="L5" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M5" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KAZBEGI-2000-PET-003. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N5">
         <v>700</v>
@@ -648,6 +696,21 @@
       </c>
       <c r="P5" t="str">
         <v>85b16a404cdffddd72a0c488b7f299e7e09420efc7b5dacfae3a0eabf52f87c5</v>
+      </c>
+      <c r="Q5" t="b">
+        <v>1</v>
+      </c>
+      <c r="R5">
+        <v>0.78</v>
+      </c>
+      <c r="S5" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="6">
@@ -672,9 +735,6 @@
       <c r="G6" t="str">
         <v>new_product</v>
       </c>
-      <c r="H6" t="str">
-        <v/>
-      </c>
       <c r="I6" t="str">
         <v/>
       </c>
@@ -685,10 +745,10 @@
         <v/>
       </c>
       <c r="L6" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M6" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KAZBEGI-2000-PET-004. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N6">
         <v>600</v>
@@ -698,6 +758,21 @@
       </c>
       <c r="P6" t="str">
         <v>9fdcaa5ad41059c963af436f0f1864932c5e0381beece86e4c63b597862559b0</v>
+      </c>
+      <c r="Q6" t="b">
+        <v>1</v>
+      </c>
+      <c r="R6">
+        <v>0.78</v>
+      </c>
+      <c r="S6" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="7">
@@ -722,9 +797,6 @@
       <c r="G7" t="str">
         <v>new_product</v>
       </c>
-      <c r="H7" t="str">
-        <v/>
-      </c>
       <c r="I7" t="str">
         <v/>
       </c>
@@ -735,10 +807,10 @@
         <v/>
       </c>
       <c r="L7" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M7" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DENEB-450-CAN-001. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N7">
         <v>1280</v>
@@ -748,6 +820,21 @@
       </c>
       <c r="P7" t="str">
         <v>ea3e58677bdcb1bbc2e1af3b05752646bd3f6af14792add98f0bdf56106cc278</v>
+      </c>
+      <c r="Q7" t="b">
+        <v>1</v>
+      </c>
+      <c r="R7">
+        <v>0.78</v>
+      </c>
+      <c r="S7" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="8">
@@ -785,10 +872,10 @@
         <v>Мохито Fresh клубника, 0,45 л, жестяная банка</v>
       </c>
       <c r="L8" t="str">
-        <v>pending</v>
+        <v>needs_review</v>
       </c>
       <c r="M8" t="str">
-        <v/>
+        <v>Авто: статус probable_match требует ручной проверки</v>
       </c>
       <c r="N8">
         <v>1280</v>
@@ -798,6 +885,21 @@
       </c>
       <c r="P8" t="str">
         <v>c1a0297b0b41326e8a38140aff53a2a172d527647136ebcc9850e69bd9f28179</v>
+      </c>
+      <c r="Q8" t="b">
+        <v>1</v>
+      </c>
+      <c r="R8">
+        <v>0.55</v>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v>status_probable_match</v>
+      </c>
+      <c r="U8" t="str">
+        <v>needs_review_probable_match</v>
       </c>
     </row>
     <row r="9">
@@ -822,9 +924,6 @@
       <c r="G9" t="str">
         <v>new_product</v>
       </c>
-      <c r="H9" t="str">
-        <v/>
-      </c>
       <c r="I9" t="str">
         <v/>
       </c>
@@ -835,10 +934,10 @@
         <v/>
       </c>
       <c r="L9" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M9" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KINZA-320-CAN-001. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N9">
         <v>680</v>
@@ -848,6 +947,21 @@
       </c>
       <c r="P9" t="str">
         <v>0b2234c7c30ad8107ad222c55ad02f2416c882f0aba835e9a3b87fd0f04e7bb6</v>
+      </c>
+      <c r="Q9" t="b">
+        <v>1</v>
+      </c>
+      <c r="R9">
+        <v>0.78</v>
+      </c>
+      <c r="S9" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="10">
@@ -885,10 +999,10 @@
         <v>Добрый Манго-маракуйя, 1 л, ПЭТ</v>
       </c>
       <c r="L10" t="str">
-        <v>pending</v>
+        <v>approved_existing</v>
       </c>
       <c r="M10" t="str">
-        <v/>
+        <v>Авто: exact_match, бренд/объём/упаковка/вкус/sugar совпали, score≥80, уникальный TINDA, фото≥500. Визуальное соответствие предполагается по exact_match — желательна выборочная ручная проверка.</v>
       </c>
       <c r="N10">
         <v>1254</v>
@@ -898,6 +1012,21 @@
       </c>
       <c r="P10" t="str">
         <v>d8c2a0353ca2d82f3439e7f66ce04ba0e639dbec18707849e3a465a5abbb7608</v>
+      </c>
+      <c r="Q10" t="b">
+        <v>1</v>
+      </c>
+      <c r="R10">
+        <v>0.82</v>
+      </c>
+      <c r="S10" t="str">
+        <v>match_status_exact|brand|volume|package|flavor_overlap_1.00|sugar_unknown|score_90|size_ge_500|image_opens|no_watermark_detected</v>
+      </c>
+      <c r="T10" t="str">
+        <v/>
+      </c>
+      <c r="U10" t="str">
+        <v>approved_existing_strict_exact</v>
       </c>
     </row>
     <row r="11">
@@ -935,10 +1064,10 @@
         <v>Добрый Манго-маракуйя, 1,5 л, ПЭТ</v>
       </c>
       <c r="L11" t="str">
-        <v>pending</v>
+        <v>approved_existing</v>
       </c>
       <c r="M11" t="str">
-        <v/>
+        <v>Авто: exact_match, бренд/объём/упаковка/вкус/sugar совпали, score≥80, уникальный TINDA, фото≥500. Визуальное соответствие предполагается по exact_match — желательна выборочная ручная проверка.</v>
       </c>
       <c r="N11">
         <v>680</v>
@@ -948,6 +1077,21 @@
       </c>
       <c r="P11" t="str">
         <v>1a3d2853c34beebad6c90e90d95774aaf0ed5dfc77cad97a0e6fe82e535b4bf9</v>
+      </c>
+      <c r="Q11" t="b">
+        <v>1</v>
+      </c>
+      <c r="R11">
+        <v>0.82</v>
+      </c>
+      <c r="S11" t="str">
+        <v>match_status_exact|brand|volume|package|flavor_overlap_1.00|sugar_unknown|score_90|size_ge_500|image_opens|no_watermark_detected</v>
+      </c>
+      <c r="T11" t="str">
+        <v/>
+      </c>
+      <c r="U11" t="str">
+        <v>approved_existing_strict_exact</v>
       </c>
     </row>
     <row r="12">
@@ -985,10 +1129,10 @@
         <v>Добрый Манго-маракуйя, 0,5 л, ПЭТ</v>
       </c>
       <c r="L12" t="str">
-        <v>pending</v>
+        <v>approved_existing</v>
       </c>
       <c r="M12" t="str">
-        <v/>
+        <v>Авто: exact_match, бренд/объём/упаковка/вкус/sugar совпали, score≥80, уникальный TINDA, фото≥500. Визуальное соответствие предполагается по exact_match — желательна выборочная ручная проверка.</v>
       </c>
       <c r="N12">
         <v>1000</v>
@@ -998,6 +1142,21 @@
       </c>
       <c r="P12" t="str">
         <v>12a3e3b2375208d095e97219bbcdaef6b93fb0aad6daf584d09b7b4ec4270d53</v>
+      </c>
+      <c r="Q12" t="b">
+        <v>1</v>
+      </c>
+      <c r="R12">
+        <v>0.82</v>
+      </c>
+      <c r="S12" t="str">
+        <v>match_status_exact|brand|volume|package|flavor_overlap_1.00|sugar_unknown|score_90|size_ge_500|image_opens|no_watermark_detected</v>
+      </c>
+      <c r="T12" t="str">
+        <v/>
+      </c>
+      <c r="U12" t="str">
+        <v>approved_existing_strict_exact</v>
       </c>
     </row>
     <row r="13">
@@ -1035,10 +1194,10 @@
         <v>Добрый Лимон-лайм, 1,5 л, ПЭТ</v>
       </c>
       <c r="L13" t="str">
-        <v>pending</v>
+        <v>approved_existing</v>
       </c>
       <c r="M13" t="str">
-        <v/>
+        <v>Авто: exact_match, бренд/объём/упаковка/вкус/sugar совпали, score≥80, уникальный TINDA, фото≥500. Визуальное соответствие предполагается по exact_match — желательна выборочная ручная проверка.</v>
       </c>
       <c r="N13">
         <v>1254</v>
@@ -1048,6 +1207,21 @@
       </c>
       <c r="P13" t="str">
         <v>51230ccebcd59d39930b2bf3a31262445db9c85fd946ad8fb2b8f3827761fc96</v>
+      </c>
+      <c r="Q13" t="b">
+        <v>1</v>
+      </c>
+      <c r="R13">
+        <v>0.82</v>
+      </c>
+      <c r="S13" t="str">
+        <v>match_status_exact|brand|volume|package|flavor_overlap_0.67|sugar_unknown|score_83|size_ge_500|image_opens|no_watermark_detected</v>
+      </c>
+      <c r="T13" t="str">
+        <v/>
+      </c>
+      <c r="U13" t="str">
+        <v>approved_existing_strict_exact</v>
       </c>
     </row>
     <row r="14">
@@ -1085,10 +1259,10 @@
         <v>Добрый Кола Ваниль, 1,5 л, ПЭТ</v>
       </c>
       <c r="L14" t="str">
-        <v>pending</v>
+        <v>needs_review</v>
       </c>
       <c r="M14" t="str">
-        <v/>
+        <v>Авто: статус conflict требует ручной проверки</v>
       </c>
       <c r="N14">
         <v>1254</v>
@@ -1098,6 +1272,21 @@
       </c>
       <c r="P14" t="str">
         <v>95127fb0c842d5f2ff52e287e24f75a6c5f22043997ea34f24454aac394b6643</v>
+      </c>
+      <c r="Q14" t="b">
+        <v>1</v>
+      </c>
+      <c r="R14">
+        <v>0.55</v>
+      </c>
+      <c r="S14" t="str">
+        <v/>
+      </c>
+      <c r="T14" t="str">
+        <v>status_conflict</v>
+      </c>
+      <c r="U14" t="str">
+        <v>needs_review_conflict</v>
       </c>
     </row>
     <row r="15">
@@ -1122,9 +1311,6 @@
       <c r="G15" t="str">
         <v>new_product</v>
       </c>
-      <c r="H15" t="str">
-        <v/>
-      </c>
       <c r="I15" t="str">
         <v/>
       </c>
@@ -1135,10 +1321,10 @@
         <v/>
       </c>
       <c r="L15" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M15" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DENEB-450-CAN-003. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N15">
         <v>1280</v>
@@ -1148,6 +1334,21 @@
       </c>
       <c r="P15" t="str">
         <v>b0d87c3dc4cee2513d56db38cf91df4d62a72ba40eeebdb5e3bce10630c4c7d3</v>
+      </c>
+      <c r="Q15" t="b">
+        <v>1</v>
+      </c>
+      <c r="R15">
+        <v>0.78</v>
+      </c>
+      <c r="S15" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T15" t="str">
+        <v/>
+      </c>
+      <c r="U15" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="16">
@@ -1172,9 +1373,6 @@
       <c r="G16" t="str">
         <v>new_product</v>
       </c>
-      <c r="H16" t="str">
-        <v/>
-      </c>
       <c r="I16" t="str">
         <v/>
       </c>
@@ -1185,10 +1383,10 @@
         <v/>
       </c>
       <c r="L16" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M16" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DENEB-450-CAN-004. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N16">
         <v>1280</v>
@@ -1198,6 +1396,21 @@
       </c>
       <c r="P16" t="str">
         <v>740992bebd8e2a1ef47ed4fff3573ba9314fca754c5603e7d779485b81fe92a1</v>
+      </c>
+      <c r="Q16" t="b">
+        <v>1</v>
+      </c>
+      <c r="R16">
+        <v>0.78</v>
+      </c>
+      <c r="S16" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T16" t="str">
+        <v/>
+      </c>
+      <c r="U16" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="17">
@@ -1222,9 +1435,6 @@
       <c r="G17" t="str">
         <v>new_product</v>
       </c>
-      <c r="H17" t="str">
-        <v/>
-      </c>
       <c r="I17" t="str">
         <v/>
       </c>
@@ -1235,10 +1445,10 @@
         <v/>
       </c>
       <c r="L17" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M17" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KINZA-320-CAN-002. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N17">
         <v>500</v>
@@ -1248,6 +1458,21 @@
       </c>
       <c r="P17" t="str">
         <v>f0f0dc1dbd221e800a21602648c6429fc14f49fc95b125f6701280e0c553f226</v>
+      </c>
+      <c r="Q17" t="b">
+        <v>1</v>
+      </c>
+      <c r="R17">
+        <v>0.78</v>
+      </c>
+      <c r="S17" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T17" t="str">
+        <v/>
+      </c>
+      <c r="U17" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="18">
@@ -1285,10 +1510,10 @@
         <v>Rich bitter Гранат, 1 л, ПЭТ</v>
       </c>
       <c r="L18" t="str">
-        <v>pending</v>
+        <v>needs_review</v>
       </c>
       <c r="M18" t="str">
-        <v/>
+        <v>Авто: статус conflict требует ручной проверки</v>
       </c>
       <c r="N18">
         <v>1254</v>
@@ -1298,6 +1523,21 @@
       </c>
       <c r="P18" t="str">
         <v>83e55bebcd9348f37e31e763256940c4d703c3f6c8a1f03124ed6d7b775264f2</v>
+      </c>
+      <c r="Q18" t="b">
+        <v>1</v>
+      </c>
+      <c r="R18">
+        <v>0.55</v>
+      </c>
+      <c r="S18" t="str">
+        <v/>
+      </c>
+      <c r="T18" t="str">
+        <v>status_conflict</v>
+      </c>
+      <c r="U18" t="str">
+        <v>needs_review_conflict</v>
       </c>
     </row>
     <row r="19">
@@ -1335,10 +1575,10 @@
         <v>Evervess Кола, 1 л, ПЭТ</v>
       </c>
       <c r="L19" t="str">
-        <v>pending</v>
+        <v>needs_review</v>
       </c>
       <c r="M19" t="str">
-        <v/>
+        <v>Авто: статус probable_match требует ручной проверки</v>
       </c>
       <c r="N19">
         <v>636</v>
@@ -1348,6 +1588,21 @@
       </c>
       <c r="P19" t="str">
         <v>78b3b7f4544ee095a330cd85c6d6a148683a3fca615445c23a1972a99df63576</v>
+      </c>
+      <c r="Q19" t="b">
+        <v>1</v>
+      </c>
+      <c r="R19">
+        <v>0.55</v>
+      </c>
+      <c r="S19" t="str">
+        <v/>
+      </c>
+      <c r="T19" t="str">
+        <v>status_probable_match</v>
+      </c>
+      <c r="U19" t="str">
+        <v>needs_review_probable_match</v>
       </c>
     </row>
     <row r="20">
@@ -1372,9 +1627,6 @@
       <c r="G20" t="str">
         <v>new_product</v>
       </c>
-      <c r="H20" t="str">
-        <v/>
-      </c>
       <c r="I20" t="str">
         <v/>
       </c>
@@ -1385,10 +1637,10 @@
         <v/>
       </c>
       <c r="L20" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M20" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KINZA-320-CAN-003. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N20">
         <v>950</v>
@@ -1398,6 +1650,21 @@
       </c>
       <c r="P20" t="str">
         <v>9b48d7c3d040ddfa23b30413750fe063ada7e1c1f5b2982f457f716717ac253e</v>
+      </c>
+      <c r="Q20" t="b">
+        <v>1</v>
+      </c>
+      <c r="R20">
+        <v>0.78</v>
+      </c>
+      <c r="S20" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T20" t="str">
+        <v/>
+      </c>
+      <c r="U20" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="21">
@@ -1422,9 +1689,6 @@
       <c r="G21" t="str">
         <v>new_product</v>
       </c>
-      <c r="H21" t="str">
-        <v/>
-      </c>
       <c r="I21" t="str">
         <v/>
       </c>
@@ -1435,10 +1699,10 @@
         <v/>
       </c>
       <c r="L21" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M21" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KINZA-320-CAN-004. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N21">
         <v>835</v>
@@ -1448,6 +1712,21 @@
       </c>
       <c r="P21" t="str">
         <v>6442890c811265bf2aace519044c2fa6c5c01ddd539237e3df4f70314dffd217</v>
+      </c>
+      <c r="Q21" t="b">
+        <v>1</v>
+      </c>
+      <c r="R21">
+        <v>0.78</v>
+      </c>
+      <c r="S21" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T21" t="str">
+        <v/>
+      </c>
+      <c r="U21" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="22">
@@ -1472,9 +1751,6 @@
       <c r="G22" t="str">
         <v>new_product</v>
       </c>
-      <c r="H22" t="str">
-        <v/>
-      </c>
       <c r="I22" t="str">
         <v/>
       </c>
@@ -1485,10 +1761,10 @@
         <v/>
       </c>
       <c r="L22" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M22" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KINZA-320-CAN-005. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N22">
         <v>750</v>
@@ -1498,6 +1774,21 @@
       </c>
       <c r="P22" t="str">
         <v>8d03db2920b4dde76741db83eabeb2c55a7de182e6a659329f882a42ec6efcd4</v>
+      </c>
+      <c r="Q22" t="b">
+        <v>1</v>
+      </c>
+      <c r="R22">
+        <v>0.78</v>
+      </c>
+      <c r="S22" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_sugar_free</v>
+      </c>
+      <c r="T22" t="str">
+        <v/>
+      </c>
+      <c r="U22" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="23">
@@ -1522,9 +1813,6 @@
       <c r="G23" t="str">
         <v>new_product</v>
       </c>
-      <c r="H23" t="str">
-        <v/>
-      </c>
       <c r="I23" t="str">
         <v/>
       </c>
@@ -1535,10 +1823,10 @@
         <v/>
       </c>
       <c r="L23" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M23" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-BORZHOMI-330-CAN-001. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N23">
         <v>1254</v>
@@ -1548,6 +1836,21 @@
       </c>
       <c r="P23" t="str">
         <v>a584fdea0dde3b7f9b33b129def10a15aecb3d289e1b092e464db6abc6ccd164</v>
+      </c>
+      <c r="Q23" t="b">
+        <v>1</v>
+      </c>
+      <c r="R23">
+        <v>0.78</v>
+      </c>
+      <c r="S23" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T23" t="str">
+        <v/>
+      </c>
+      <c r="U23" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="24">
@@ -1572,9 +1875,6 @@
       <c r="G24" t="str">
         <v>new_product</v>
       </c>
-      <c r="H24" t="str">
-        <v/>
-      </c>
       <c r="I24" t="str">
         <v/>
       </c>
@@ -1585,10 +1885,10 @@
         <v/>
       </c>
       <c r="L24" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M24" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-BORZHOMI-330-CAN-002. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N24">
         <v>1254</v>
@@ -1598,6 +1898,21 @@
       </c>
       <c r="P24" t="str">
         <v>8bcf0385713bb7f9173304b2ff3b96cb3c6fc343174b6316055924bc2dcad2ba</v>
+      </c>
+      <c r="Q24" t="b">
+        <v>1</v>
+      </c>
+      <c r="R24">
+        <v>0.78</v>
+      </c>
+      <c r="S24" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T24" t="str">
+        <v/>
+      </c>
+      <c r="U24" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="25">
@@ -1635,10 +1950,10 @@
         <v>Добрый Кола, 0,25 л, стекло</v>
       </c>
       <c r="L25" t="str">
-        <v>pending</v>
+        <v>needs_review</v>
       </c>
       <c r="M25" t="str">
-        <v/>
+        <v>Авто: статус probable_match требует ручной проверки</v>
       </c>
       <c r="N25">
         <v>1000</v>
@@ -1648,6 +1963,21 @@
       </c>
       <c r="P25" t="str">
         <v>34b9f84dfec8c812dc7f809883f60fac03b21f93d264901ebb0d534f2169e0b4</v>
+      </c>
+      <c r="Q25" t="b">
+        <v>1</v>
+      </c>
+      <c r="R25">
+        <v>0.55</v>
+      </c>
+      <c r="S25" t="str">
+        <v/>
+      </c>
+      <c r="T25" t="str">
+        <v>status_probable_match</v>
+      </c>
+      <c r="U25" t="str">
+        <v>needs_review_probable_match</v>
       </c>
     </row>
     <row r="26">
@@ -1672,9 +2002,6 @@
       <c r="G26" t="str">
         <v>new_product</v>
       </c>
-      <c r="H26" t="str">
-        <v/>
-      </c>
       <c r="I26" t="str">
         <v/>
       </c>
@@ -1685,10 +2012,10 @@
         <v/>
       </c>
       <c r="L26" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M26" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-TBILISSIMO-500-GLASS-001. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N26">
         <v>984</v>
@@ -1698,6 +2025,21 @@
       </c>
       <c r="P26" t="str">
         <v>7f3cc472ea76f2fd601a0921d048eb3d80f84a102f7d2d26f6bad063816abb06</v>
+      </c>
+      <c r="Q26" t="b">
+        <v>1</v>
+      </c>
+      <c r="R26">
+        <v>0.78</v>
+      </c>
+      <c r="S26" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T26" t="str">
+        <v/>
+      </c>
+      <c r="U26" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="27">
@@ -1722,9 +2064,6 @@
       <c r="G27" t="str">
         <v>new_product</v>
       </c>
-      <c r="H27" t="str">
-        <v/>
-      </c>
       <c r="I27" t="str">
         <v/>
       </c>
@@ -1735,10 +2074,10 @@
         <v/>
       </c>
       <c r="L27" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M27" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KINZA-320-CAN-006. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N27">
         <v>500</v>
@@ -1748,6 +2087,21 @@
       </c>
       <c r="P27" t="str">
         <v>9dc42ae0d6c3a5b77e57f5202620f11d2bd199ba1ae0c6c512a150cd464b9821</v>
+      </c>
+      <c r="Q27" t="b">
+        <v>1</v>
+      </c>
+      <c r="R27">
+        <v>0.78</v>
+      </c>
+      <c r="S27" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T27" t="str">
+        <v/>
+      </c>
+      <c r="U27" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="28">
@@ -1772,9 +2126,6 @@
       <c r="G28" t="str">
         <v>new_product</v>
       </c>
-      <c r="H28" t="str">
-        <v/>
-      </c>
       <c r="I28" t="str">
         <v/>
       </c>
@@ -1785,10 +2136,10 @@
         <v/>
       </c>
       <c r="L28" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M28" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KINZA-320-CAN-007. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N28">
         <v>800</v>
@@ -1798,6 +2149,21 @@
       </c>
       <c r="P28" t="str">
         <v>26a42bc19faae9e9fa7b39b60cc64aced952d097fc7819e27df806afd4ba00f6</v>
+      </c>
+      <c r="Q28" t="b">
+        <v>1</v>
+      </c>
+      <c r="R28">
+        <v>0.78</v>
+      </c>
+      <c r="S28" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T28" t="str">
+        <v/>
+      </c>
+      <c r="U28" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="29">
@@ -1835,10 +2201,10 @@
         <v>Добрый Кола, 0,3 л, ПЭТ</v>
       </c>
       <c r="L29" t="str">
-        <v>pending</v>
+        <v>needs_review</v>
       </c>
       <c r="M29" t="str">
-        <v/>
+        <v>Авто: exact_match, но не все строгие условия (rival_tinda_count_1)</v>
       </c>
       <c r="N29">
         <v>800</v>
@@ -1848,6 +2214,21 @@
       </c>
       <c r="P29" t="str">
         <v>effab1fcf1afd9eb512a8b6d5cb50cd40988bd9556baff3fbd1497672ec017d6</v>
+      </c>
+      <c r="Q29" t="b">
+        <v>1</v>
+      </c>
+      <c r="R29">
+        <v>0.6</v>
+      </c>
+      <c r="S29" t="str">
+        <v>match_status_exact|brand|volume|package|flavor_overlap_1.00|sugar_unknown|score_90|size_ge_500|image_opens|no_watermark_detected</v>
+      </c>
+      <c r="T29" t="str">
+        <v>rival_tinda_count_1</v>
+      </c>
+      <c r="U29" t="str">
+        <v>needs_review_exact_incomplete</v>
       </c>
     </row>
     <row r="30">
@@ -1885,10 +2266,10 @@
         <v>Добрый Кола без сахара, 0,3 л, ПЭТ</v>
       </c>
       <c r="L30" t="str">
-        <v>pending</v>
+        <v>needs_review</v>
       </c>
       <c r="M30" t="str">
-        <v/>
+        <v>Авто: статус probable_match требует ручной проверки</v>
       </c>
       <c r="N30">
         <v>800</v>
@@ -1898,6 +2279,21 @@
       </c>
       <c r="P30" t="str">
         <v>3e4a2ef52c199c0d2da14d23c209ed186d32db58d35370cdeaa9ddc357c1e567</v>
+      </c>
+      <c r="Q30" t="b">
+        <v>1</v>
+      </c>
+      <c r="R30">
+        <v>0.55</v>
+      </c>
+      <c r="S30" t="str">
+        <v/>
+      </c>
+      <c r="T30" t="str">
+        <v>status_probable_match</v>
+      </c>
+      <c r="U30" t="str">
+        <v>needs_review_probable_match</v>
       </c>
     </row>
     <row r="31">
@@ -1922,9 +2318,6 @@
       <c r="G31" t="str">
         <v>new_product</v>
       </c>
-      <c r="H31" t="str">
-        <v/>
-      </c>
       <c r="I31" t="str">
         <v/>
       </c>
@@ -1935,10 +2328,10 @@
         <v/>
       </c>
       <c r="L31" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M31" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KOLA-1500-PET-001. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N31">
         <v>900</v>
@@ -1948,6 +2341,21 @@
       </c>
       <c r="P31" t="str">
         <v>91c74d178c76201138bb5f75f99299a32ddd941e588fa5c487b9e87539e19c6c</v>
+      </c>
+      <c r="Q31" t="b">
+        <v>1</v>
+      </c>
+      <c r="R31">
+        <v>0.78</v>
+      </c>
+      <c r="S31" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match|marked_regular</v>
+      </c>
+      <c r="T31" t="str">
+        <v/>
+      </c>
+      <c r="U31" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="32">
@@ -1985,10 +2393,10 @@
         <v>Добрый Апельсин, 1 л, ПЭТ</v>
       </c>
       <c r="L32" t="str">
-        <v>pending</v>
+        <v>needs_review</v>
       </c>
       <c r="M32" t="str">
-        <v/>
+        <v>Авто: статус conflict требует ручной проверки</v>
       </c>
       <c r="N32">
         <v>418</v>
@@ -1998,6 +2406,21 @@
       </c>
       <c r="P32" t="str">
         <v>0f54d1774f575921ec0a2b3affbc9eb75ae720c4806cb8f3e9b677892e7739cc</v>
+      </c>
+      <c r="Q32" t="b">
+        <v>1</v>
+      </c>
+      <c r="R32">
+        <v>0.55</v>
+      </c>
+      <c r="S32" t="str">
+        <v/>
+      </c>
+      <c r="T32" t="str">
+        <v>status_conflict|below_500</v>
+      </c>
+      <c r="U32" t="str">
+        <v>needs_review_conflict</v>
       </c>
     </row>
     <row r="33">
@@ -2022,9 +2445,6 @@
       <c r="G33" t="str">
         <v>new_product</v>
       </c>
-      <c r="H33" t="str">
-        <v/>
-      </c>
       <c r="I33" t="str">
         <v/>
       </c>
@@ -2035,10 +2455,10 @@
         <v/>
       </c>
       <c r="L33" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M33" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-TBILISSIMO-500-GLASS-002. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N33">
         <v>796</v>
@@ -2048,6 +2468,21 @@
       </c>
       <c r="P33" t="str">
         <v>941566da675c527c77e381f49185a978b28d6dcf7b5ddeac36d476b4e260e44c</v>
+      </c>
+      <c r="Q33" t="b">
+        <v>1</v>
+      </c>
+      <c r="R33">
+        <v>0.78</v>
+      </c>
+      <c r="S33" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T33" t="str">
+        <v/>
+      </c>
+      <c r="U33" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="34">
@@ -2085,10 +2520,10 @@
         <v>Добрый Лимон-лайм, 0,5 л, ПЭТ</v>
       </c>
       <c r="L34" t="str">
-        <v>pending</v>
+        <v>approved_existing</v>
       </c>
       <c r="M34" t="str">
-        <v/>
+        <v>Авто: exact_match, бренд/объём/упаковка/вкус/sugar совпали, score≥80, уникальный TINDA, фото≥500. Визуальное соответствие предполагается по exact_match — желательна выборочная ручная проверка.</v>
       </c>
       <c r="N34">
         <v>680</v>
@@ -2098,6 +2533,21 @@
       </c>
       <c r="P34" t="str">
         <v>5ad24e8c755791a07006fca921d540766c9f841702ecb9503a698b394024c401</v>
+      </c>
+      <c r="Q34" t="b">
+        <v>1</v>
+      </c>
+      <c r="R34">
+        <v>0.82</v>
+      </c>
+      <c r="S34" t="str">
+        <v>match_status_exact|brand|volume|package|flavor_overlap_0.67|sugar_unknown|score_83|size_ge_500|image_opens|no_watermark_detected</v>
+      </c>
+      <c r="T34" t="str">
+        <v/>
+      </c>
+      <c r="U34" t="str">
+        <v>approved_existing_strict_exact</v>
       </c>
     </row>
     <row r="35">
@@ -2122,9 +2572,6 @@
       <c r="G35" t="str">
         <v>new_product</v>
       </c>
-      <c r="H35" t="str">
-        <v/>
-      </c>
       <c r="I35" t="str">
         <v/>
       </c>
@@ -2135,10 +2582,10 @@
         <v/>
       </c>
       <c r="L35" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M35" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-TBILISSIMO-500-GLASS-003. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N35">
         <v>672</v>
@@ -2148,6 +2595,21 @@
       </c>
       <c r="P35" t="str">
         <v>2dcee1d8c8242f67e4fab90b612431871c00da14e6aa49d230d970003de0f8e8</v>
+      </c>
+      <c r="Q35" t="b">
+        <v>1</v>
+      </c>
+      <c r="R35">
+        <v>0.78</v>
+      </c>
+      <c r="S35" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T35" t="str">
+        <v/>
+      </c>
+      <c r="U35" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="36">
@@ -2172,9 +2634,6 @@
       <c r="G36" t="str">
         <v>new_product</v>
       </c>
-      <c r="H36" t="str">
-        <v/>
-      </c>
       <c r="I36" t="str">
         <v/>
       </c>
@@ -2185,10 +2644,10 @@
         <v/>
       </c>
       <c r="L36" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M36" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-TBILISSIMO-500-GLASS-004. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N36">
         <v>851</v>
@@ -2198,6 +2657,21 @@
       </c>
       <c r="P36" t="str">
         <v>927def55224aa3a2453d27ecea4396850890d33dba5202747d0b63c82078d767</v>
+      </c>
+      <c r="Q36" t="b">
+        <v>1</v>
+      </c>
+      <c r="R36">
+        <v>0.78</v>
+      </c>
+      <c r="S36" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T36" t="str">
+        <v/>
+      </c>
+      <c r="U36" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="37">
@@ -2222,9 +2696,6 @@
       <c r="G37" t="str">
         <v>new_product</v>
       </c>
-      <c r="H37" t="str">
-        <v/>
-      </c>
       <c r="I37" t="str">
         <v/>
       </c>
@@ -2235,10 +2706,10 @@
         <v/>
       </c>
       <c r="L37" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M37" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-DRPEPPER-330-CAN-001. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N37">
         <v>1024</v>
@@ -2248,6 +2719,21 @@
       </c>
       <c r="P37" t="str">
         <v>487dbcb4c64c81f84d994aba49c261f4fafc462ead0e503d4e8006136b2374c8</v>
+      </c>
+      <c r="Q37" t="b">
+        <v>1</v>
+      </c>
+      <c r="R37">
+        <v>0.78</v>
+      </c>
+      <c r="S37" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T37" t="str">
+        <v/>
+      </c>
+      <c r="U37" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="38">
@@ -2272,9 +2758,6 @@
       <c r="G38" t="str">
         <v>new_product</v>
       </c>
-      <c r="H38" t="str">
-        <v/>
-      </c>
       <c r="I38" t="str">
         <v/>
       </c>
@@ -2285,10 +2768,10 @@
         <v/>
       </c>
       <c r="L38" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M38" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SWAG-330-GLASS-001. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N38">
         <v>1024</v>
@@ -2298,6 +2781,21 @@
       </c>
       <c r="P38" t="str">
         <v>ac29d6cf5b69b9402b5e70efa645b208fdd11531b110977a0188a74137a58dee</v>
+      </c>
+      <c r="Q38" t="b">
+        <v>1</v>
+      </c>
+      <c r="R38">
+        <v>0.78</v>
+      </c>
+      <c r="S38" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T38" t="str">
+        <v/>
+      </c>
+      <c r="U38" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="39">
@@ -2322,9 +2820,6 @@
       <c r="G39" t="str">
         <v>new_product</v>
       </c>
-      <c r="H39" t="str">
-        <v/>
-      </c>
       <c r="I39" t="str">
         <v/>
       </c>
@@ -2335,10 +2830,10 @@
         <v/>
       </c>
       <c r="L39" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M39" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-SWAG-330-GLASS-002. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N39">
         <v>1024</v>
@@ -2348,6 +2843,21 @@
       </c>
       <c r="P39" t="str">
         <v>bfd3f2f7fa2412964d3feeead7a4294746d958ff131c0bc7d9506c7d94307208</v>
+      </c>
+      <c r="Q39" t="b">
+        <v>1</v>
+      </c>
+      <c r="R39">
+        <v>0.78</v>
+      </c>
+      <c r="S39" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T39" t="str">
+        <v/>
+      </c>
+      <c r="U39" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="40">
@@ -2385,10 +2895,10 @@
         <v>Frustyle лимон-лайм, 1,5 л, ПЭТ</v>
       </c>
       <c r="L40" t="str">
-        <v>pending</v>
+        <v>approved_existing</v>
       </c>
       <c r="M40" t="str">
-        <v/>
+        <v>Авто: exact_match, бренд/объём/упаковка/вкус/sugar совпали, score≥80, уникальный TINDA, фото≥500. Визуальное соответствие предполагается по exact_match — желательна выборочная ручная проверка.</v>
       </c>
       <c r="N40">
         <v>1024</v>
@@ -2398,6 +2908,21 @@
       </c>
       <c r="P40" t="str">
         <v>86059b3dd786c96d85de76717483484be3419e978733974669b3b4447d165963</v>
+      </c>
+      <c r="Q40" t="b">
+        <v>1</v>
+      </c>
+      <c r="R40">
+        <v>0.82</v>
+      </c>
+      <c r="S40" t="str">
+        <v>match_status_exact|brand|volume|package|flavor_overlap_0.67|sugar_unknown|score_83|size_ge_500|image_opens|no_watermark_detected</v>
+      </c>
+      <c r="T40" t="str">
+        <v/>
+      </c>
+      <c r="U40" t="str">
+        <v>approved_existing_strict_exact</v>
       </c>
     </row>
     <row r="41">
@@ -2435,10 +2960,10 @@
         <v>Frustyle апельсин, 1,5 л, ПЭТ</v>
       </c>
       <c r="L41" t="str">
-        <v>pending</v>
+        <v>approved_existing</v>
       </c>
       <c r="M41" t="str">
-        <v/>
+        <v>Авто: exact_match, бренд/объём/упаковка/вкус/sugar совпали, score≥80, уникальный TINDA, фото≥500. Визуальное соответствие предполагается по exact_match — желательна выборочная ручная проверка.</v>
       </c>
       <c r="N41">
         <v>1024</v>
@@ -2448,6 +2973,21 @@
       </c>
       <c r="P41" t="str">
         <v>a50e9abf2ff4e1562b04cd4b93773b89439af9f7d37afe54923e9c4857d92582</v>
+      </c>
+      <c r="Q41" t="b">
+        <v>1</v>
+      </c>
+      <c r="R41">
+        <v>0.82</v>
+      </c>
+      <c r="S41" t="str">
+        <v>match_status_exact|brand|volume|package|flavor_overlap_0.50|sugar_unknown|score_83|size_ge_500|image_opens|no_watermark_detected</v>
+      </c>
+      <c r="T41" t="str">
+        <v/>
+      </c>
+      <c r="U41" t="str">
+        <v>approved_existing_strict_exact</v>
       </c>
     </row>
     <row r="42">
@@ -2472,9 +3012,6 @@
       <c r="G42" t="str">
         <v>new_product</v>
       </c>
-      <c r="H42" t="str">
-        <v/>
-      </c>
       <c r="I42" t="str">
         <v/>
       </c>
@@ -2485,10 +3022,10 @@
         <v/>
       </c>
       <c r="L42" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M42" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-FRUSTAIL-330-CAN-001. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N42">
         <v>1024</v>
@@ -2498,6 +3035,21 @@
       </c>
       <c r="P42" t="str">
         <v>9cfaae610f76c9ee281fcd1256faee5e73460b27999e66458b01068f5ac7f8bc</v>
+      </c>
+      <c r="Q42" t="b">
+        <v>1</v>
+      </c>
+      <c r="R42">
+        <v>0.78</v>
+      </c>
+      <c r="S42" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T42" t="str">
+        <v/>
+      </c>
+      <c r="U42" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="43">
@@ -2535,10 +3087,10 @@
         <v>Добрый Лимон-лайм, 1 л, ПЭТ</v>
       </c>
       <c r="L43" t="str">
-        <v>pending</v>
+        <v>approved_existing</v>
       </c>
       <c r="M43" t="str">
-        <v/>
+        <v>Авто: exact_match, бренд/объём/упаковка/вкус/sugar совпали, score≥80, уникальный TINDA, фото≥500. Визуальное соответствие предполагается по exact_match — желательна выборочная ручная проверка.</v>
       </c>
       <c r="N43">
         <v>1024</v>
@@ -2548,6 +3100,21 @@
       </c>
       <c r="P43" t="str">
         <v>25176b344a0b6b750e176004531bc231fc78a229fd7f5f9a915028efe61c18d0</v>
+      </c>
+      <c r="Q43" t="b">
+        <v>1</v>
+      </c>
+      <c r="R43">
+        <v>0.82</v>
+      </c>
+      <c r="S43" t="str">
+        <v>match_status_exact|brand|volume|package|flavor_overlap_0.67|sugar_unknown|score_83|size_ge_500|image_opens|no_watermark_detected</v>
+      </c>
+      <c r="T43" t="str">
+        <v/>
+      </c>
+      <c r="U43" t="str">
+        <v>approved_existing_strict_exact</v>
       </c>
     </row>
     <row r="44">
@@ -2585,10 +3152,10 @@
         <v>Добрый Лимон-лайм, 0,33 л, жестяная банка</v>
       </c>
       <c r="L44" t="str">
-        <v>pending</v>
+        <v>approved_existing</v>
       </c>
       <c r="M44" t="str">
-        <v/>
+        <v>Авто: exact_match, бренд/объём/упаковка/вкус/sugar совпали, score≥80, уникальный TINDA, фото≥500. Визуальное соответствие предполагается по exact_match — желательна выборочная ручная проверка.</v>
       </c>
       <c r="N44">
         <v>1254</v>
@@ -2598,6 +3165,21 @@
       </c>
       <c r="P44" t="str">
         <v>8711152d221d8a15afe945e747b34083745f7634b56308a9829f504b1b143761</v>
+      </c>
+      <c r="Q44" t="b">
+        <v>1</v>
+      </c>
+      <c r="R44">
+        <v>0.82</v>
+      </c>
+      <c r="S44" t="str">
+        <v>match_status_exact|brand|volume|package|flavor_overlap_0.67|sugar_unknown|score_83|size_ge_500|image_opens|no_watermark_detected</v>
+      </c>
+      <c r="T44" t="str">
+        <v/>
+      </c>
+      <c r="U44" t="str">
+        <v>approved_existing_strict_exact</v>
       </c>
     </row>
     <row r="45">
@@ -2622,9 +3204,6 @@
       <c r="G45" t="str">
         <v>new_product</v>
       </c>
-      <c r="H45" t="str">
-        <v/>
-      </c>
       <c r="I45" t="str">
         <v/>
       </c>
@@ -2635,10 +3214,10 @@
         <v/>
       </c>
       <c r="L45" t="str">
-        <v>pending</v>
+        <v>needs_review</v>
       </c>
       <c r="M45" t="str">
-        <v/>
+        <v>Авто: изображение меньше 500×500</v>
       </c>
       <c r="N45">
         <v>200</v>
@@ -2648,6 +3227,21 @@
       </c>
       <c r="P45" t="str">
         <v>f2a9cac3ddf1ca803bbe83c1b7f0c2f4f38ddff37120e1be583fbff56b2229cd</v>
+      </c>
+      <c r="Q45" t="b">
+        <v>1</v>
+      </c>
+      <c r="R45">
+        <v>0.7</v>
+      </c>
+      <c r="S45" t="str">
+        <v/>
+      </c>
+      <c r="T45" t="str">
+        <v>below_500</v>
+      </c>
+      <c r="U45" t="str">
+        <v>needs_review_small_image</v>
       </c>
     </row>
     <row r="46">
@@ -2685,10 +3279,10 @@
         <v>Добрый Апельсин, 0,5 л, ПЭТ</v>
       </c>
       <c r="L46" t="str">
-        <v>pending</v>
+        <v>needs_review</v>
       </c>
       <c r="M46" t="str">
-        <v/>
+        <v>Авто: статус conflict требует ручной проверки</v>
       </c>
       <c r="N46">
         <v>1024</v>
@@ -2698,6 +3292,21 @@
       </c>
       <c r="P46" t="str">
         <v>9a39dd1b2b6d48d1410a79002e1818ef1a7d79d5ec5093a9ccf51c272200ca80</v>
+      </c>
+      <c r="Q46" t="b">
+        <v>1</v>
+      </c>
+      <c r="R46">
+        <v>0.55</v>
+      </c>
+      <c r="S46" t="str">
+        <v/>
+      </c>
+      <c r="T46" t="str">
+        <v>status_conflict</v>
+      </c>
+      <c r="U46" t="str">
+        <v>needs_review_conflict</v>
       </c>
     </row>
     <row r="47">
@@ -2735,10 +3344,10 @@
         <v>Добрый Кола, 0,33 л, жестяная банка</v>
       </c>
       <c r="L47" t="str">
-        <v>pending</v>
+        <v>needs_review</v>
       </c>
       <c r="M47" t="str">
-        <v/>
+        <v>Авто: статус probable_match требует ручной проверки</v>
       </c>
       <c r="N47">
         <v>1024</v>
@@ -2748,6 +3357,21 @@
       </c>
       <c r="P47" t="str">
         <v>051010e4eadd05d76eb9210476063d6ccb94140aacfc09a6b9fee676619a0c26</v>
+      </c>
+      <c r="Q47" t="b">
+        <v>1</v>
+      </c>
+      <c r="R47">
+        <v>0.55</v>
+      </c>
+      <c r="S47" t="str">
+        <v/>
+      </c>
+      <c r="T47" t="str">
+        <v>status_probable_match</v>
+      </c>
+      <c r="U47" t="str">
+        <v>needs_review_probable_match</v>
       </c>
     </row>
     <row r="48">
@@ -2772,9 +3396,6 @@
       <c r="G48" t="str">
         <v>new_product</v>
       </c>
-      <c r="H48" t="str">
-        <v/>
-      </c>
       <c r="I48" t="str">
         <v/>
       </c>
@@ -2785,10 +3406,10 @@
         <v/>
       </c>
       <c r="L48" t="str">
-        <v>pending</v>
+        <v>approved_new</v>
       </c>
       <c r="M48" t="str">
-        <v/>
+        <v>Авто: new_product, атрибуты распознаны, нет near-дубля в ТИНДА, фото≥500. proposed_sku=ZY-KAZBEGI-500-GLASS-001. Товар ещё не создан — только кандидат.</v>
       </c>
       <c r="N48">
         <v>1024</v>
@@ -2798,6 +3419,21 @@
       </c>
       <c r="P48" t="str">
         <v>42b2c834371329ea7c02405d0339cf99e852a2d0eb719ccd226a81062b394563</v>
+      </c>
+      <c r="Q48" t="b">
+        <v>1</v>
+      </c>
+      <c r="R48">
+        <v>0.78</v>
+      </c>
+      <c r="S48" t="str">
+        <v>brand_parsed|name_present|flavor_present|volume_parsed|package_parsed|size_ge_500|image_opens|no_watermark_detected|no_tinda_near_match</v>
+      </c>
+      <c r="T48" t="str">
+        <v/>
+      </c>
+      <c r="U48" t="str">
+        <v>approved_new_clean_candidate</v>
       </c>
     </row>
     <row r="49">
@@ -2822,9 +3458,6 @@
       <c r="G49" t="str">
         <v>new_product</v>
       </c>
-      <c r="H49" t="str">
-        <v/>
-      </c>
       <c r="I49" t="str">
         <v/>
       </c>
@@ -2835,10 +3468,10 @@
         <v/>
       </c>
       <c r="L49" t="str">
-        <v>pending</v>
+        <v>rejected</v>
       </c>
       <c r="M49" t="str">
-        <v/>
+        <v>Авто: placeholder / слишком маленький файл</v>
       </c>
       <c r="N49">
         <v>225</v>
@@ -2849,10 +3482,25 @@
       <c r="P49" t="str">
         <v>b2f140edc8d4c200121e4914cf7477629ebfd41a5200dfb4da7208965b33bcc8</v>
       </c>
+      <c r="Q49" t="b">
+        <v>1</v>
+      </c>
+      <c r="R49">
+        <v>0.85</v>
+      </c>
+      <c r="S49" t="str">
+        <v/>
+      </c>
+      <c r="T49" t="str">
+        <v>placeholder_like|file_size_3680</v>
+      </c>
+      <c r="U49" t="str">
+        <v>rejected_placeholder</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P49"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U49"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2874,7 +3522,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Локальный review. Не загружать на VPS и не менять image_url автоматически.</v>
+        <v>Автоматическая предварительная проверка. Требует ручной выборочной валидации.</v>
       </c>
     </row>
     <row r="3">
@@ -2882,7 +3530,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>review_status: pending | approved_existing | approved_new | rejected</v>
+        <v>Не загружать на VPS и не менять image_url автоматически.</v>
       </c>
     </row>
   </sheetData>

</xml_diff>